<commit_message>
planning out plant stuff
</commit_message>
<xml_diff>
--- a/xlsx/HerbalNames.xlsx
+++ b/xlsx/HerbalNames.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hadle\Documents\GitHub\voynichTEI\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8854C489-692C-49B4-850C-4C0FC1BCDEBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB26D0FC-0093-4AE1-8144-D7277F21A44E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E74B4125-5874-4082-9055-372A93C35FC0}"/>
+    <workbookView xWindow="-108" yWindow="672" windowWidth="11664" windowHeight="11952" xr2:uid="{E74B4125-5874-4082-9055-372A93C35FC0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>